<commit_message>
Enhance run.bat and Streamlit configuration for improved development experience
- Updated `run.bat` to automatically close any previous instances running on port 8501 before starting Streamlit, ensuring a smoother development workflow.
- Modified `.streamlit/config.toml` to enable automatic app reload on code changes, set the server to run in headless mode, and adjusted browser settings for local development.
</commit_message>
<xml_diff>
--- a/exports/informe_cliente_2026-07-01_2026-07-07.xlsx
+++ b/exports/informe_cliente_2026-07-01_2026-07-07.xlsx
@@ -21,8 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00&quot; €&quot;"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,16 +32,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B1F3A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +59,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E6EC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E6EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E6EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E6EC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -127,6 +171,71 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaInformeEvolucion" displayName="TablaInformeEvolucion" ref="A1:E6" headerRowCount="1">
+  <autoFilter ref="A1:E6"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Fecha"/>
+    <tableColumn id="2" name="Consumo"/>
+    <tableColumn id="3" name="Merma"/>
+    <tableColumn id="4" name="Expiración"/>
+    <tableColumn id="5" name="Total"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TablaInformeDesayunos" displayName="TablaInformeDesayunos" ref="A1:D5" headerRowCount="1">
+  <autoFilter ref="A1:D5"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Fecha"/>
+    <tableColumn id="2" name="Huéspedes"/>
+    <tableColumn id="3" name="Coste"/>
+    <tableColumn id="4" name="Registrado por"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TablaInformeMermas" displayName="TablaInformeMermas" ref="A1:C7" headerRowCount="1">
+  <autoFilter ref="A1:C7"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Fecha"/>
+    <tableColumn id="2" name="Coste"/>
+    <tableColumn id="3" name="Registrado por"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TablaInformeInventario" displayName="TablaInformeInventario" ref="A1:D11" headerRowCount="1">
+  <autoFilter ref="A1:D11"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Producto"/>
+    <tableColumn id="2" name="Unidad"/>
+    <tableColumn id="3" name="Stock"/>
+    <tableColumn id="4" name="Stock mínimo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TablaInformeAlertas" displayName="TablaInformeAlertas" ref="A1:D10" headerRowCount="1">
+  <autoFilter ref="A1:D10"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Título"/>
+    <tableColumn id="2" name="Mensaje"/>
+    <tableColumn id="3" name="Tipo"/>
+    <tableColumn id="4" name="Fecha"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -420,127 +529,131 @@
   </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Establecimiento</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Hotel Boutique La Alameda</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Royal Marina Suites</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Informe</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Resumen operativo de desayuno</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Periodo desde</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>01/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Periodo hasta</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Generado</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>07/07/2026 17:34</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 20:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Coste total</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>60.17</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="B7" s="3" t="n">
+        <v>62.37</v>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Coste consumo</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>41.67</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="B8" s="3" t="n">
+        <v>43.87</v>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Coste merma</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>10.9</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Coste expiración</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="3" t="n">
         <v>7.6</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Coste por huésped</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>2.005666666666667</v>
+      <c r="B11" s="3" t="n">
+        <v>2.079</v>
       </c>
     </row>
   </sheetData>
@@ -556,131 +669,141 @@
   </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Consumo</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Merma</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Expiración</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="6" t="n">
         <v>0.6</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="6" t="n">
         <v>0.6</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>04/07/2026</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="6" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="6" t="n">
         <v>10.52</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="6" t="n">
         <v>15.25</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="6" t="n">
         <v>15.25</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="6" t="n">
         <v>16.8</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="6" t="n">
         <v>17.8</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
+      <c r="B6" s="6" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E6" t="n">
-        <v>16</v>
+      <c r="E6" s="6" t="n">
+        <v>18.2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -690,66 +813,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Huéspedes</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Coste</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Registrado por</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>María García</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="C3" s="6" t="n">
         <v>16.8</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B4" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="C4" s="6" t="n">
         <v>15.25</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>04/07/2026</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B5" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C5" s="6" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Carlos Ruiz</t>
         </is>
@@ -757,6 +918,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -768,109 +932,114 @@
   </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Coste</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Registrado por</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="6" t="n">
         <v>5.5</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>04/07/2026</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Carlos Ruiz</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="6" t="n">
         <v>0.6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
@@ -878,6 +1047,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -889,211 +1061,220 @@
   </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Stock mínimo</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Café molido</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Kg</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Croissant</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Fruta fresca</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Huevos</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Jamón serrano</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Mantequilla</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
         <v>0.3</v>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Croissant</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="D7" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Pan de molde</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Ud</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>42</v>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Fruta fresca</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="C8" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Queso manchego</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Kg</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Huevos</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="C9" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Yogur natural</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Ud</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Jamón serrano</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mantequilla</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Pan de molde</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Ud</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="C10" s="5" t="n">
         <v>10</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Queso manchego</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Kg</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Yogur natural</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Ud</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="D10" s="5" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Zumo de naranja</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="5" t="n">
         <v>4.5</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="5" t="n">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1103,334 +1284,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Título</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Mensaje</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Merma superior al mes anterior</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>La merma acumulada supera un 15% respecto al mes pasado.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>merma_elevada</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Revisar proveedor de jamón</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Verificar precio del próximo pedido con Embutidos Norte.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Stock bajo — Pan de molde</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Quedan 8 Ud. Stock mínimo: 10.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Stock bajo — Yogur natural</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Quedan 10 Ud. Stock mínimo: 24.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>stock_bajo</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Stock bajo — Jamón serrano</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Quedan 1.2 Kg. Stock mínimo: 2.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Stock bajo — Zumo de naranja</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Quedan 4.5 L. Stock mínimo: 5.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>stock_bajo</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Stock bajo — Queso manchego</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Quedan 0.6 Kg. Stock mínimo: 1.5.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Stock bajo — Café molido</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Quedan 0.1 Kg. Stock mínimo: 1.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>stock_bajo</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Stock bajo — Yogur natural</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Quedan 10 Ud. Stock mínimo: 24.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Stock bajo — Mantequilla</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Quedan 0.3 Kg. Stock mínimo: 0.5.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>stock_bajo</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Stock bajo — Zumo de naranja</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Quedan 4.5 L. Stock mínimo: 5.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Stock bajo — Fruta fresca</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Quedan 2.1 Kg. Stock mínimo: 3.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>stock_bajo</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Stock bajo — Café molido</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Quedan 0.3 Kg. Stock mínimo: 1.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>stock_bajo</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Stock agotado — Huevos</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>No quedan unidades disponibles.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>stock_cero</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Stock bajo — Mantequilla</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Quedan 0.3 Kg. Stock mínimo: 0.5.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>stock_bajo</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Próximo a expirar — Croissant</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>El lote l01 (compra 02/07/2026) expira en 3 día(s).</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>expiracion_proxima</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Stock bajo — Fruta fresca</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Quedan 2.1 Kg. Stock mínimo: 3.</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>stock_bajo</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Stock agotado — Huevos</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>No quedan unidades disponibles.</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>stock_cero</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Próximo a expirar — Croissant</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>El lote l01 (compra 02/07/2026) expira en 3 día(s).</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Próximo a expirar — Yogur natural</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>El lote l05 (compra 03/07/2026) expira en 2 día(s).</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>expiracion_proxima</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Próximo a expirar — Yogur natural</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>El lote l05 (compra 03/07/2026) expira en 2 día(s).</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>expiracion_proxima</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Desayuno de hoy no registrado</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Aún no se ha registrado el consumo del desayuno de hoy.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>desayuno_no_registrado</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
@@ -1438,5 +1515,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>